<commit_message>
Se agrega en localstorage grupos terapeuticos de clave a partir de CPM
</commit_message>
<xml_diff>
--- a/public/template_abasto.xlsx
+++ b/public/template_abasto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\solicitudes-app\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892DA8EB-A925-4B80-AF20-8347492C5C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{571DF9D3-E617-434D-AD7C-B2155BC3A98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>#</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>Total piezas disponibles:</t>
+  </si>
+  <si>
+    <t>Grupo</t>
+  </si>
+  <si>
+    <t>Gpo Terapéutico</t>
   </si>
 </sst>
 </file>
@@ -634,13 +640,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="11" width="15" customWidth="1"/>
+    <col min="1" max="1" width="4.5703125" customWidth="1"/>
+    <col min="2" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="18.28515625" customWidth="1"/>
+    <col min="8" max="13" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -657,21 +666,27 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix al reporte estatal
</commit_message>
<xml_diff>
--- a/public/template_abasto.xlsx
+++ b/public/template_abasto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\solicitudes-app\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469CF7DF-1D97-4847-8A86-97AE70401330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C739DF87-DEAD-4D44-97D5-9CFED468CCC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,7 +80,7 @@
     <t>Ordenes recibidas ultimos 40 dias</t>
   </si>
   <si>
-    <t>Obvservaciones</t>
+    <t>Observaciones</t>
   </si>
 </sst>
 </file>
@@ -654,7 +654,7 @@
     <col min="7" max="7" width="18.28515625" customWidth="1"/>
     <col min="8" max="13" width="15" customWidth="1"/>
     <col min="14" max="14" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="37" customWidth="1"/>
+    <col min="15" max="15" width="99.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>